<commit_message>
docs(extraction): retire les tirets cadratins du canevas et de la spec DAP
Remplace tiret cadratin/demi-cadratin/signe moins par une ponctuation
équivalente (« · », deux-points, parenthèses, trait d'union simple) dans
le gabarit Canevas_Extraction_mSupply_DQA_v2.xlsx (onglets MODE_EMPLOI,
SITES, SITE_PROGRAMME, PRODUITS, TRANSACTIONS, LIGNES_TRANSACTIONS) et
dans docs/specification_extraction_dap.md, avant envoi à la DAP.

Le classeur est reconstruit avec des séparateurs '/' conformes OOXML
(Compress-Archive et System.IO.Compression.ZipFile utilisent '\' sur
Windows) ; relu par le pipeline d'import réel pour vérifier la lisibilité.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Canevas_Extraction_mSupply_DQA_v2.xlsx
+++ b/docs/Canevas_Extraction_mSupply_DQA_v2.xlsx
@@ -147,7 +147,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">CANEVAS D'EXTRACTION mSupply — TABLEAU DE BORD DQA</t>
+          <t xml:space="preserve">CANEVAS D'EXTRACTION mSupply · TABLEAU DE BORD DQA</t>
         </is>
       </c>
       <c r="B1" s="0"/>
@@ -155,7 +155,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nouvelle PSP-CI / DAP — Spécification v2.0 (2026-08-28)</t>
+          <t xml:space="preserve">Nouvelle PSP-CI / DAP · Spécification v2.0 (2026-08-28)</t>
         </is>
       </c>
       <c r="B2" s="0"/>
@@ -256,7 +256,7 @@
       <c r="A17" s="0"/>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 mois consécutifs, notés M+1 à M+4. Trois cycles par an sur l'année civile : C1 janvier–avril, C2 mai–août, C3 septembre–décembre.</t>
+          <t xml:space="preserve">4 mois consécutifs, notés M+1 à M+4. Trois cycles par an sur l'année civile : C1 janvier-avril, C2 mai-août, C3 septembre-décembre.</t>
         </is>
       </c>
     </row>
@@ -422,7 +422,7 @@
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Détail produit des transactions — PRODUITS TRACEURS UNIQUEMENT.</t>
+          <t xml:space="preserve">Détail produit des transactions (PRODUITS TRACEURS UNIQUEMENT).</t>
         </is>
       </c>
     </row>
@@ -434,7 +434,7 @@
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stock disponible à la date d'extraction — TRACEURS UNIQUEMENT.</t>
+          <t xml:space="preserve">Stock disponible à la date d'extraction (TRACEURS UNIQUEMENT).</t>
         </is>
       </c>
     </row>
@@ -458,7 +458,7 @@
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Détail produit des inventaires — TRACEURS UNIQUEMENT, sans doublon.</t>
+          <t xml:space="preserve">Détail produit des inventaires (TRACEURS UNIQUEMENT, sans doublon).</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">INVENTAIRE_LIGNES — une ligne (inventaire, produit, lot). TRACEURS UNIQUEMENT. Une seule ligne par clé, sans doublon.</t>
+          <t xml:space="preserve">INVENTAIRE_LIGNES · une ligne (inventaire, produit, lot). TRACEURS UNIQUEMENT. Une seule ligne par clé, sans doublon.</t>
         </is>
       </c>
     </row>
@@ -718,7 +718,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">REQUISITIONS — une réquisition. Fenêtre = date_entered ou période couverte touchant la fenêtre.</t>
+          <t xml:space="preserve">REQUISITIONS · une réquisition. Fenêtre = date_entered ou période couverte touchant la fenêtre.</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1240,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SITES — un site (magasin mSupply). Inclure tous les magasins actifs.</t>
+          <t xml:space="preserve">SITES · un site (magasin mSupply). Inclure tous les magasins actifs.</t>
         </is>
       </c>
     </row>
@@ -1250,7 +1250,7 @@
     <row r="4" ht="135" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obligatoire. store.id — identifiant mSupply du magasin.</t>
+          <t xml:space="preserve">Obligatoire. store.id (identifiant mSupply du magasin).</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -1414,7 +1414,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SITE_PROGRAMME — un couple (site, programme géré). Pilote le pilier P1.</t>
+          <t xml:space="preserve">SITE_PROGRAMME · un couple (site, programme géré). Pilote le pilier P1.</t>
         </is>
       </c>
     </row>
@@ -1528,7 +1528,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PRODUITS — un produit. Tous les produits (le marquage traceur est géré côté tableau de bord).</t>
+          <t xml:space="preserve">PRODUITS · un produit. Tous les produits (le marquage traceur est géré côté tableau de bord).</t>
         </is>
       </c>
     </row>
@@ -1651,7 +1651,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRANSACTIONS — une transaction (en-tête). Fenêtre = confirm_date ou finalised_date dans la fenêtre.</t>
+          <t xml:space="preserve">TRANSACTIONS · une transaction (en-tête). Fenêtre = confirm_date ou finalised_date dans la fenêtre.</t>
         </is>
       </c>
     </row>
@@ -1671,7 +1671,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obligatoire. Valeur dérivée — voir §5.1 de la spécification. Valeurs : dispensation, distribution, facture_fournisseur, reception, ajustement_positif, ajustement_negatif, retour_fournisseur, retour_client, autre.</t>
+          <t xml:space="preserve">Obligatoire. Valeur dérivée (voir §5.1 de la spécification). Valeurs : dispensation, distribution, facture_fournisseur, reception, ajustement_positif, ajustement_negatif, retour_fournisseur, retour_client, autre.</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -1901,7 +1901,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">LIGNES_TRANSACTIONS — une ligne (transaction, produit, lot). PRODUITS TRACEURS UNIQUEMENT.</t>
+          <t xml:space="preserve">LIGNES_TRANSACTIONS · une ligne (transaction, produit, lot). PRODUITS TRACEURS UNIQUEMENT.</t>
         </is>
       </c>
     </row>
@@ -1936,12 +1936,12 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obligatoire. trans_line.quantity — quantité réelle en conditionnement.</t>
+          <t xml:space="preserve">Obligatoire. trans_line.quantity (quantité réelle en conditionnement).</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obligatoire. trans_line.pack_size — unités de dispensation par conditionnement.</t>
+          <t xml:space="preserve">Obligatoire. trans_line.pack_size (unités de dispensation par conditionnement).</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -2091,7 +2091,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">STOCK_ACTUEL — un lot en stock (site, produit, lot) à la date d'extraction. TRACEURS UNIQUEMENT.</t>
+          <t xml:space="preserve">STOCK_ACTUEL · un lot en stock (site, produit, lot) à la date d'extraction. TRACEURS UNIQUEMENT.</t>
         </is>
       </c>
     </row>
@@ -2222,7 +2222,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">INVENTAIRES — un inventaire (stock_take, en-tête). Fenêtre = stock_take_date dans la fenêtre.</t>
+          <t xml:space="preserve">INVENTAIRES · un inventaire (stock_take, en-tête). Fenêtre = stock_take_date dans la fenêtre.</t>
         </is>
       </c>
     </row>

</xml_diff>